<commit_message>
Tactical Fulton Extraction System 업데이트
Co-Authored-By: DeaD DooDle <33118840+basalt991@users.noreply.github.com>

#2897
</commit_message>
<xml_diff>
--- a/Data/Tactical Fulton Extraction System - 3687327231/1.6/3687327231.xlsx
+++ b/Data/Tactical Fulton Extraction System - 3687327231/1.6/3687327231.xlsx
@@ -8,7 +8,8 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Main_260321" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Current_260409" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="260321" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="66">
   <si>
     <t xml:space="preserve">Class+Node [(Identifier (Key)]</t>
   </si>
@@ -35,6 +36,138 @@
   </si>
   <si>
     <t xml:space="preserve">English [Source string]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Korean (한국어) [Translation]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResearchProjectDef+FultonExtractionTech.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResearchProjectDef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FultonExtractionTech.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fulton extraction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">풀톤 회수 시스템</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResearchProjectDef+FultonExtractionTech.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FultonExtractionTech.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advanced tactical recovery systems using high-pressure balloons and specialized logistics crates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고압 풍선을 이용해 인원과 특별 수송 상자를 신속히 회수하는 기술입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JobDef+Fulton_ExtractJob.reportString</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JobDef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fulton_ExtractJob.reportString</t>
+  </si>
+  <si>
+    <t xml:space="preserve">extracting Target.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">대상 회수 중</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+FultonHarness.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FultonHarness.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fulton extraction harness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">풀톤 회수 하네스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+FultonHarness.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FultonHarness.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A tactical recovery system. Can be used to extract pawns, items, and buildings to your home map. Note: Hostile humans and wild animals must be knocked out before they can be attached to the balloon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전술 회수 장비입니다. 사람, 물품, 건물을 본거지 맵으로 회수할 수 있습니다. 참고: 적대적인 인간과 야생 동물은 풍선에 연결하기 전에 기절한 상태여야 합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+FultonLandingPad.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FultonLandingPad.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fulton landing pad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">풀톤 착륙 패드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+FultonLandingPad.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FultonLandingPad.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A designated recovery zone for Fulton extractions. Built into the ground to allow heavy crates, items, and pawns to land safely on top of it without damaging the structure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">풀톤 회수용으로 지정된 회수 구역입니다. 지면에 매립식으로 설치되어, 무거운 상자와 물품, 인원이 구조물에 손상을 주지 않고 그 위에 안전하게 착지할 수 있도록 설계되었습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResearchTabDef+RoltonsModsTab.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResearchTabDef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RoltonsModsTab.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rolton's Mods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+FultonStorageCrate.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FultonStorageCrate.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fulton storage crate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">풀톤 수송 상자</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+FultonStorageCrate.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FultonStorageCrate.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A large receiving crate. Use the 'Extract Crate' button to air-lift the crate and EVERY item currently sitting on its tile back home. Can be uninstalled and carried on caravans.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">대형 회수용 상자입니다. ‘상자 회수’ 버튼을 사용하면, 이 상자와 현재 이 타일 위에 놓여 있는 모든 물품을 공중 회수하여 본거지로 보낼 수 있습니다. 포장하여 상단에 실어 운반할 수 있습니다.</t>
   </si>
   <si>
     <r>
@@ -53,6 +186,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">한국어</t>
     </r>
@@ -68,27 +202,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">ResearchProjectDef+FultonExtractionTech.label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ResearchProjectDef</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FultonExtractionTech.label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fulton extraction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">풀톤 회수 시스템</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ResearchProjectDef+FultonExtractionTech.description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FultonExtractionTech.description</t>
-  </si>
-  <si>
     <t xml:space="preserve">Technology to rapidly extract personnel and materials using high-pressure balloons.</t>
   </si>
   <si>
@@ -98,6 +211,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">풍선을 이용해 인원과 물자를 신속히 회수하는 기술입니다</t>
     </r>
@@ -113,15 +227,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">JobDef+Fulton_ExtractJob.reportString</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JobDef</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fulton_ExtractJob.reportString</t>
-  </si>
-  <si>
     <t xml:space="preserve">extracting TargetA.</t>
   </si>
   <si>
@@ -141,30 +246,10 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">회수 중</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">ThingDef+FultonHarness.label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ThingDef</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FultonHarness.label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fulton extraction harness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">풀톤 회수 하네스</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ThingDef+FultonHarness.description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FultonHarness.description</t>
   </si>
   <si>
     <t xml:space="preserve">A tactical recovery system. Allows targeting of pawns, items, and corpses anywhere on the map. Hostiles must be downed. Cannot be used under roofs.</t>
@@ -176,6 +261,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">전술 회수 장비입니다</t>
     </r>
@@ -195,6 +281,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">맵 어디에서든 사람</t>
     </r>
@@ -214,6 +301,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">물품</t>
     </r>
@@ -233,6 +321,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">시체를 대상으로 지정할 수 있습니다</t>
     </r>
@@ -252,6 +341,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">적대 대상은 쓰러진 상태여야 합니다</t>
     </r>
@@ -271,6 +361,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">지붕 아래에서는 사용할 수 없습니다</t>
     </r>
@@ -310,24 +401,6 @@
     <t xml:space="preserve">풀톤 풍선</t>
   </si>
   <si>
-    <t xml:space="preserve">ThingDef+FultonLandingPad.label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FultonLandingPad.label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fulton landing pad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">풀톤 착륙 패드</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ThingDef+FultonLandingPad.description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FultonLandingPad.description</t>
-  </si>
-  <si>
     <t xml:space="preserve">A tactical recovery zone. extracted targets land here.</t>
   </si>
   <si>
@@ -337,6 +410,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">전술 회수 구역입니다</t>
     </r>
@@ -356,6 +430,7 @@
         <color rgb="FF000000"/>
         <rFont val="나눔고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">회수된 대상이 이곳에 착륙합니다</t>
     </r>
@@ -384,6 +459,7 @@
       <color rgb="FF000000"/>
       <name val="나눔고딕"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -450,12 +526,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -648,188 +728,405 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:F1048576"/>
+  <sheetFormatPr defaultColWidth="12.046875" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="73.86"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,보통"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,보통"&amp;12&amp;Kffffff페이지 &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="12.046875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="39.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="67.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="7" style="0" width="7.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="39.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="67.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="7" style="1" width="7.27"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
+      <c r="F1" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>14</v>
+      <c r="E3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>19</v>
+      <c r="E4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>28</v>
+      <c r="E6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c r="A7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>32</v>
+      <c r="C7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="1" t="s">
+      <c r="A8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>36</v>
+      <c r="C8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="1" t="s">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="0" t="s">
-        <v>40</v>
+      <c r="C9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="A10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="0" t="s">
-        <v>44</v>
+      <c r="C10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>